<commit_message>
Agrega serie de irregularidad agregada y ajustes de figuras
</commit_message>
<xml_diff>
--- a/fuentes_y_definiciones.xlsx
+++ b/fuentes_y_definiciones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivanurquiza/Desktop/Cowork/NOTA-Mora_Credit/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C93AA739-4B11-144C-A3DD-31AE494A1259}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFCDFD89-5639-1243-BAA2-2C97044AC43E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16680" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Irregularidad BCRA" sheetId="1" r:id="rId1"/>
@@ -399,7 +399,7 @@
     <numFmt numFmtId="165" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="167" formatCode="_(* #,##0.000_);_(* \(#,##0.000\);_(* &quot;-&quot;???_);_(@_)"/>
-    <numFmt numFmtId="174" formatCode="0.0"/>
+    <numFmt numFmtId="168" formatCode="0.0"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -595,14 +595,8 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="14" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -612,6 +606,12 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="14" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -931,14 +931,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="32"/>
-      <c r="E1" s="32"/>
-      <c r="F1" s="33"/>
+      <c r="B1" s="36"/>
+      <c r="C1" s="36"/>
+      <c r="D1" s="37"/>
+      <c r="E1" s="37"/>
+      <c r="F1" s="38"/>
     </row>
     <row r="2" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
@@ -7232,25 +7232,25 @@
       <c r="G1" s="39"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="36" t="s">
+      <c r="A2" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="37" t="s">
+      <c r="B2" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="C2" s="37" t="s">
+      <c r="C2" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="D2" s="38" t="s">
+      <c r="D2" s="34" t="s">
         <v>37</v>
       </c>
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="F2" s="37" t="s">
+      <c r="F2" s="33" t="s">
         <v>109</v>
       </c>
-      <c r="G2" s="38" t="s">
+      <c r="G2" s="34" t="s">
         <v>38</v>
       </c>
     </row>
@@ -7266,8 +7266,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A3,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1338513185</v>
       </c>
-      <c r="D3" s="35">
-        <f t="shared" ref="D3:D26" si="0">(B3-C3)/B3*100</f>
+      <c r="D3" s="31">
+        <f>(B3-C3)/B3*100</f>
         <v>8.5119701711251121</v>
       </c>
       <c r="E3" s="29">
@@ -7278,8 +7278,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A3,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1415511473</v>
       </c>
-      <c r="G3" s="35">
-        <f t="shared" ref="G3:G26" si="1">(E3-F3)/E3*100</f>
+      <c r="G3" s="31">
+        <f t="shared" ref="G3:G26" si="0">(E3-F3)/E3*100</f>
         <v>8.0925677013033042</v>
       </c>
     </row>
@@ -7295,8 +7295,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A4,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1517432417</v>
       </c>
-      <c r="D4" s="35">
-        <f t="shared" si="0"/>
+      <c r="D4" s="31">
+        <f t="shared" ref="D3:D26" si="1">(B4-C4)/B4*100</f>
         <v>7.6821482890986221</v>
       </c>
       <c r="E4" s="29">
@@ -7307,8 +7307,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A4,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1572641042</v>
       </c>
-      <c r="G4" s="35">
-        <f t="shared" si="1"/>
+      <c r="G4" s="31">
+        <f t="shared" si="0"/>
         <v>7.4340394466379882</v>
       </c>
     </row>
@@ -7324,8 +7324,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A5,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1572094460</v>
       </c>
-      <c r="D5" s="35">
-        <f t="shared" si="0"/>
+      <c r="D5" s="31">
+        <f t="shared" si="1"/>
         <v>7.3054664824144497</v>
       </c>
       <c r="E5" s="29">
@@ -7336,8 +7336,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A5,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1623127732</v>
       </c>
-      <c r="G5" s="35">
-        <f t="shared" si="1"/>
+      <c r="G5" s="31">
+        <f t="shared" si="0"/>
         <v>7.0932431231597537</v>
       </c>
     </row>
@@ -7353,8 +7353,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A6,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1743213099</v>
       </c>
-      <c r="D6" s="35">
-        <f t="shared" si="0"/>
+      <c r="D6" s="31">
+        <f t="shared" si="1"/>
         <v>6.9580660106905574</v>
       </c>
       <c r="E6" s="29">
@@ -7365,8 +7365,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A6,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1809660143</v>
       </c>
-      <c r="G6" s="35">
-        <f t="shared" si="1"/>
+      <c r="G6" s="31">
+        <f t="shared" si="0"/>
         <v>6.720228750438249</v>
       </c>
     </row>
@@ -7382,8 +7382,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A7,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1773036838</v>
       </c>
-      <c r="D7" s="35">
-        <f t="shared" si="0"/>
+      <c r="D7" s="31">
+        <f t="shared" si="1"/>
         <v>7.2080982399953113</v>
       </c>
       <c r="E7" s="29">
@@ -7394,8 +7394,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A7,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1833069057</v>
       </c>
-      <c r="G7" s="35">
-        <f t="shared" si="1"/>
+      <c r="G7" s="31">
+        <f t="shared" si="0"/>
         <v>7.0207361618170472</v>
       </c>
     </row>
@@ -7411,8 +7411,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A8,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>1869909919</v>
       </c>
-      <c r="D8" s="35">
-        <f t="shared" si="0"/>
+      <c r="D8" s="31">
+        <f t="shared" si="1"/>
         <v>7.9232061178146536</v>
       </c>
       <c r="E8" s="29">
@@ -7423,8 +7423,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A8,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>1942995471</v>
       </c>
-      <c r="G8" s="35">
-        <f t="shared" si="1"/>
+      <c r="G8" s="31">
+        <f t="shared" si="0"/>
         <v>7.6489510606999929</v>
       </c>
     </row>
@@ -7440,8 +7440,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A9,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>2068695596</v>
       </c>
-      <c r="D9" s="35">
-        <f t="shared" si="0"/>
+      <c r="D9" s="31">
+        <f t="shared" si="1"/>
         <v>7.1784101937345506</v>
       </c>
       <c r="E9" s="29">
@@ -7452,8 +7452,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A9,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>2137504953</v>
       </c>
-      <c r="G9" s="35">
-        <f t="shared" si="1"/>
+      <c r="G9" s="31">
+        <f t="shared" si="0"/>
         <v>6.9656576671014907</v>
       </c>
     </row>
@@ -7469,8 +7469,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A10,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>2451091727</v>
       </c>
-      <c r="D10" s="35">
-        <f t="shared" si="0"/>
+      <c r="D10" s="31">
+        <f t="shared" si="1"/>
         <v>6.8579695415556738</v>
       </c>
       <c r="E10" s="29">
@@ -7481,8 +7481,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A10,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>2528115665</v>
       </c>
-      <c r="G10" s="35">
-        <f t="shared" si="1"/>
+      <c r="G10" s="31">
+        <f t="shared" si="0"/>
         <v>6.6660550397986542</v>
       </c>
     </row>
@@ -7498,8 +7498,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A11,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>2678642361</v>
       </c>
-      <c r="D11" s="35">
-        <f t="shared" si="0"/>
+      <c r="D11" s="31">
+        <f t="shared" si="1"/>
         <v>6.2673016802932926</v>
       </c>
       <c r="E11" s="29">
@@ -7510,8 +7510,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A11,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>2761434942</v>
       </c>
-      <c r="G11" s="35">
-        <f t="shared" si="1"/>
+      <c r="G11" s="31">
+        <f t="shared" si="0"/>
         <v>6.0924832052243261</v>
       </c>
     </row>
@@ -7527,8 +7527,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A12,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>3277113004</v>
       </c>
-      <c r="D12" s="35">
-        <f t="shared" si="0"/>
+      <c r="D12" s="31">
+        <f t="shared" si="1"/>
         <v>5.0783408377469001</v>
       </c>
       <c r="E12" s="29">
@@ -7539,8 +7539,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A12,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>3375562818</v>
       </c>
-      <c r="G12" s="35">
-        <f t="shared" si="1"/>
+      <c r="G12" s="31">
+        <f t="shared" si="0"/>
         <v>4.9387552849118803</v>
       </c>
     </row>
@@ -7556,8 +7556,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A13,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>3592124212</v>
       </c>
-      <c r="D13" s="35">
-        <f t="shared" si="0"/>
+      <c r="D13" s="31">
+        <f t="shared" si="1"/>
         <v>5.2342531725701296</v>
       </c>
       <c r="E13" s="29">
@@ -7568,8 +7568,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A13,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>3696338823</v>
       </c>
-      <c r="G13" s="35">
-        <f t="shared" si="1"/>
+      <c r="G13" s="31">
+        <f t="shared" si="0"/>
         <v>5.0951767272929427</v>
       </c>
     </row>
@@ -7585,8 +7585,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A14,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>4129316398</v>
       </c>
-      <c r="D14" s="35">
-        <f t="shared" si="0"/>
+      <c r="D14" s="31">
+        <f t="shared" si="1"/>
         <v>5.1972958291373041</v>
       </c>
       <c r="E14" s="29">
@@ -7597,8 +7597,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A14,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>4254075134</v>
       </c>
-      <c r="G14" s="35">
-        <f t="shared" si="1"/>
+      <c r="G14" s="31">
+        <f t="shared" si="0"/>
         <v>5.0572198067381402</v>
       </c>
     </row>
@@ -7614,8 +7614,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A15,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>4829746920</v>
       </c>
-      <c r="D15" s="35">
-        <f t="shared" si="0"/>
+      <c r="D15" s="31">
+        <f t="shared" si="1"/>
         <v>5.4087850178592838</v>
       </c>
       <c r="E15" s="29">
@@ -7626,8 +7626,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A15,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>4974999752</v>
       </c>
-      <c r="G15" s="35">
-        <f t="shared" si="1"/>
+      <c r="G15" s="31">
+        <f t="shared" si="0"/>
         <v>5.2628826865293403</v>
       </c>
     </row>
@@ -7643,8 +7643,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A16,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>6297996457</v>
       </c>
-      <c r="D16" s="35">
-        <f t="shared" si="0"/>
+      <c r="D16" s="31">
+        <f t="shared" si="1"/>
         <v>5.1432579850478586</v>
       </c>
       <c r="E16" s="29">
@@ -7655,8 +7655,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A16,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>6555618996</v>
       </c>
-      <c r="G16" s="35">
-        <f t="shared" si="1"/>
+      <c r="G16" s="31">
+        <f t="shared" si="0"/>
         <v>4.9543047505329723</v>
       </c>
     </row>
@@ -7672,8 +7672,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A17,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>8025666435</v>
       </c>
-      <c r="D17" s="35">
-        <f t="shared" si="0"/>
+      <c r="D17" s="31">
+        <f t="shared" si="1"/>
         <v>5.466110093558151</v>
       </c>
       <c r="E17" s="29">
@@ -7684,8 +7684,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A17,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>8302300875</v>
       </c>
-      <c r="G17" s="35">
-        <f t="shared" si="1"/>
+      <c r="G17" s="31">
+        <f t="shared" si="0"/>
         <v>5.2939800604385825</v>
       </c>
     </row>
@@ -7701,8 +7701,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A18,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>10759740150</v>
       </c>
-      <c r="D18" s="35">
-        <f t="shared" si="0"/>
+      <c r="D18" s="31">
+        <f t="shared" si="1"/>
         <v>6.8825511262631327</v>
       </c>
       <c r="E18" s="29">
@@ -7713,8 +7713,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A18,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>11110394313</v>
       </c>
-      <c r="G18" s="35">
-        <f t="shared" si="1"/>
+      <c r="G18" s="31">
+        <f t="shared" si="0"/>
         <v>6.6819507913600642</v>
       </c>
     </row>
@@ -7730,8 +7730,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A19,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>14787970193</v>
       </c>
-      <c r="D19" s="35">
-        <f t="shared" si="0"/>
+      <c r="D19" s="31">
+        <f t="shared" si="1"/>
         <v>3.2598592314941319</v>
       </c>
       <c r="E19" s="29">
@@ -7742,8 +7742,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A19,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>15218401152</v>
       </c>
-      <c r="G19" s="35">
-        <f t="shared" si="1"/>
+      <c r="G19" s="31">
+        <f t="shared" si="0"/>
         <v>3.1708767957426045</v>
       </c>
     </row>
@@ -7759,8 +7759,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A20,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>21455860567</v>
       </c>
-      <c r="D20" s="35">
-        <f t="shared" si="0"/>
+      <c r="D20" s="31">
+        <f t="shared" si="1"/>
         <v>2.5163662211347626</v>
       </c>
       <c r="E20" s="29">
@@ -7771,8 +7771,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A20,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>22062091846</v>
       </c>
-      <c r="G20" s="35">
-        <f t="shared" si="1"/>
+      <c r="G20" s="31">
+        <f t="shared" si="0"/>
         <v>2.4511750431324373</v>
       </c>
     </row>
@@ -7788,8 +7788,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A21,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>30644546252</v>
       </c>
-      <c r="D21" s="35">
-        <f t="shared" si="0"/>
+      <c r="D21" s="31">
+        <f t="shared" si="1"/>
         <v>1.9200661499351488</v>
       </c>
       <c r="E21" s="29">
@@ -7800,8 +7800,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A21,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>31319488391</v>
       </c>
-      <c r="G21" s="35">
-        <f t="shared" si="1"/>
+      <c r="G21" s="31">
+        <f t="shared" si="0"/>
         <v>1.8863696360274074</v>
       </c>
     </row>
@@ -7817,8 +7817,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A22,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>40168920828</v>
       </c>
-      <c r="D22" s="35">
-        <f t="shared" si="0"/>
+      <c r="D22" s="31">
+        <f t="shared" si="1"/>
         <v>1.9515918099971923</v>
       </c>
       <c r="E22" s="29">
@@ -7829,8 +7829,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A22,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>40907617306</v>
       </c>
-      <c r="G22" s="35">
-        <f t="shared" si="1"/>
+      <c r="G22" s="31">
+        <f t="shared" si="0"/>
         <v>1.9175939649271139</v>
       </c>
     </row>
@@ -7846,8 +7846,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A23,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>48555620291</v>
       </c>
-      <c r="D23" s="35">
-        <f t="shared" si="0"/>
+      <c r="D23" s="31">
+        <f t="shared" si="1"/>
         <v>2.5955112550506509</v>
       </c>
       <c r="E23" s="29">
@@ -7858,8 +7858,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A23,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>49455902270</v>
       </c>
-      <c r="G23" s="35">
-        <f t="shared" si="1"/>
+      <c r="G23" s="31">
+        <f t="shared" si="0"/>
         <v>2.5573882049992496</v>
       </c>
     </row>
@@ -7875,8 +7875,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A24,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>58407031679</v>
       </c>
-      <c r="D24" s="35">
-        <f t="shared" si="0"/>
+      <c r="D24" s="31">
+        <f t="shared" si="1"/>
         <v>2.7845493769290202</v>
       </c>
       <c r="E24" s="29">
@@ -7887,8 +7887,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A24,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>59538502281</v>
       </c>
-      <c r="G24" s="35">
-        <f t="shared" si="1"/>
+      <c r="G24" s="31">
+        <f t="shared" si="0"/>
         <v>2.738907925347585</v>
       </c>
     </row>
@@ -7904,8 +7904,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A25,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>65164537912</v>
       </c>
-      <c r="D25" s="35">
-        <f t="shared" si="0"/>
+      <c r="D25" s="31">
+        <f t="shared" si="1"/>
         <v>4.0987039948796991</v>
       </c>
       <c r="E25" s="29">
@@ -7916,8 +7916,8 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A25,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>66296591313</v>
       </c>
-      <c r="G25" s="35">
-        <f t="shared" si="1"/>
+      <c r="G25" s="31">
+        <f t="shared" si="0"/>
         <v>4.0323747702046484</v>
       </c>
     </row>
@@ -7933,8 +7933,8 @@
         <f>SUMIFS('Irregularidad BCRA'!$E$3:$E$314,'Irregularidad BCRA'!$A$3:$A$314,A26,'Irregularidad BCRA'!$B$3:$B$314,"&lt;&gt;L")</f>
         <v>71199272617</v>
       </c>
-      <c r="D26" s="35">
-        <f t="shared" si="0"/>
+      <c r="D26" s="31">
+        <f t="shared" si="1"/>
         <v>4.589784544776383</v>
       </c>
       <c r="E26" s="29">
@@ -7945,21 +7945,21 @@
         <f>SUMIF('Irregularidad BCRA'!$A$3:$A$314,A26,'Irregularidad BCRA'!$E$3:$E$314)</f>
         <v>72513539219</v>
       </c>
-      <c r="G26" s="35">
-        <f t="shared" si="1"/>
+      <c r="G26" s="31">
+        <f t="shared" si="0"/>
         <v>4.6086011048877262</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B27" s="35"/>
-      <c r="C27" s="35"/>
-      <c r="D27" s="35"/>
-      <c r="E27" s="35"/>
-      <c r="F27" s="35"/>
-      <c r="G27" s="35"/>
+      <c r="B27" s="31"/>
+      <c r="C27" s="31"/>
+      <c r="D27" s="31"/>
+      <c r="E27" s="31"/>
+      <c r="F27" s="31"/>
+      <c r="G27" s="31"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A28" s="34"/>
+      <c r="A28" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>